<commit_message>
Rename three columns: 2026 Proj Pts, 2025 Pts, Conf Lvl
Pts -> 2026 Proj Pts, 2025 Exp PPG -> 2025 Pts, Conf -> Conf Lvl.
Applied to the HTML board and all 7 workbook tabs, plus the prose in the
README and the workbook's Settings notes, so the two artifacts and the
docs describe the same column names.

Dropping "EXP PPG" fixes one misreading and risks another: the header no
longer wrongly claims a per-game figure, but "2025 Pts" now reads as a raw
season total, and it isn't one -- Allen scored 159 in 2025 and the column
shows 178.9, his rate over a full 18 games. The header tooltip now says so
explicitly rather than leaving it implied.

Workbook formulas reference cell letters, not header text, so nothing
recalculates differently. Verified headers on both outputs after rebuild.
</commit_message>
<xml_diff>
--- a/2026 TD-FG League Draft Board.xlsx
+++ b/2026 TD-FG League Draft Board.xlsx
@@ -584,11 +584,11 @@
     <col width="6" customWidth="1" min="10" max="10"/>
     <col width="7" customWidth="1" min="11" max="11"/>
     <col width="6" customWidth="1" min="12" max="12"/>
-    <col width="9" customWidth="1" min="13" max="13"/>
+    <col width="11" customWidth="1" min="13" max="13"/>
     <col width="10" customWidth="1" min="14" max="14"/>
     <col width="8" customWidth="1" min="15" max="15"/>
     <col width="9" customWidth="1" min="16" max="16"/>
-    <col width="8" customWidth="1" min="17" max="17"/>
+    <col width="9" customWidth="1" min="17" max="17"/>
     <col width="62" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
@@ -662,12 +662,12 @@
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>Points</t>
+          <t>2026 Proj Pts</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>2025 Exp</t>
+          <t>2025 Pts</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
@@ -682,7 +682,7 @@
       </c>
       <c r="Q2" s="2" t="inlineStr">
         <is>
-          <t>Conf</t>
+          <t>Conf Lvl</t>
         </is>
       </c>
       <c r="R2" s="2" t="inlineStr">
@@ -18083,7 +18083,7 @@
     <row r="22">
       <c r="F22" s="23" t="inlineStr">
         <is>
-          <t>tab and Points/VOR/Adj VOR recalculate.</t>
+          <t>tab and 2026 Proj Pts / VOR / Adj VOR recalculate.</t>
         </is>
       </c>
     </row>
@@ -18093,7 +18093,7 @@
     <row r="24">
       <c r="F24" s="23" t="inlineStr">
         <is>
-          <t>2025 Exp is not a projection and not editable: it is what the player actually scored</t>
+          <t>2025 Pts is not a projection and not editable: it is what the player actually scored</t>
         </is>
       </c>
     </row>
@@ -18158,11 +18158,11 @@
     <col width="6" customWidth="1" min="10" max="10"/>
     <col width="7" customWidth="1" min="11" max="11"/>
     <col width="6" customWidth="1" min="12" max="12"/>
-    <col width="9" customWidth="1" min="13" max="13"/>
+    <col width="11" customWidth="1" min="13" max="13"/>
     <col width="10" customWidth="1" min="14" max="14"/>
     <col width="8" customWidth="1" min="15" max="15"/>
     <col width="9" customWidth="1" min="16" max="16"/>
-    <col width="8" customWidth="1" min="17" max="17"/>
+    <col width="9" customWidth="1" min="17" max="17"/>
     <col width="62" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
@@ -18236,12 +18236,12 @@
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>Points</t>
+          <t>2026 Proj Pts</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>2025 Exp</t>
+          <t>2025 Pts</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
@@ -18256,7 +18256,7 @@
       </c>
       <c r="Q2" s="2" t="inlineStr">
         <is>
-          <t>Conf</t>
+          <t>Conf Lvl</t>
         </is>
       </c>
       <c r="R2" s="2" t="inlineStr">
@@ -20484,11 +20484,11 @@
     <col width="6" customWidth="1" min="10" max="10"/>
     <col width="7" customWidth="1" min="11" max="11"/>
     <col width="6" customWidth="1" min="12" max="12"/>
-    <col width="9" customWidth="1" min="13" max="13"/>
+    <col width="11" customWidth="1" min="13" max="13"/>
     <col width="10" customWidth="1" min="14" max="14"/>
     <col width="8" customWidth="1" min="15" max="15"/>
     <col width="9" customWidth="1" min="16" max="16"/>
-    <col width="8" customWidth="1" min="17" max="17"/>
+    <col width="9" customWidth="1" min="17" max="17"/>
     <col width="62" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
@@ -20562,12 +20562,12 @@
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>Points</t>
+          <t>2026 Proj Pts</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>2025 Exp</t>
+          <t>2025 Pts</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
@@ -20582,7 +20582,7 @@
       </c>
       <c r="Q2" s="2" t="inlineStr">
         <is>
-          <t>Conf</t>
+          <t>Conf Lvl</t>
         </is>
       </c>
       <c r="R2" s="2" t="inlineStr">
@@ -24779,11 +24779,11 @@
     <col width="6" customWidth="1" min="10" max="10"/>
     <col width="7" customWidth="1" min="11" max="11"/>
     <col width="6" customWidth="1" min="12" max="12"/>
-    <col width="9" customWidth="1" min="13" max="13"/>
+    <col width="11" customWidth="1" min="13" max="13"/>
     <col width="10" customWidth="1" min="14" max="14"/>
     <col width="8" customWidth="1" min="15" max="15"/>
     <col width="9" customWidth="1" min="16" max="16"/>
-    <col width="8" customWidth="1" min="17" max="17"/>
+    <col width="9" customWidth="1" min="17" max="17"/>
     <col width="62" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
@@ -24857,12 +24857,12 @@
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>Points</t>
+          <t>2026 Proj Pts</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>2025 Exp</t>
+          <t>2025 Pts</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
@@ -24877,7 +24877,7 @@
       </c>
       <c r="Q2" s="2" t="inlineStr">
         <is>
-          <t>Conf</t>
+          <t>Conf Lvl</t>
         </is>
       </c>
       <c r="R2" s="2" t="inlineStr">
@@ -29657,11 +29657,11 @@
     <col width="6" customWidth="1" min="10" max="10"/>
     <col width="7" customWidth="1" min="11" max="11"/>
     <col width="6" customWidth="1" min="12" max="12"/>
-    <col width="9" customWidth="1" min="13" max="13"/>
+    <col width="11" customWidth="1" min="13" max="13"/>
     <col width="10" customWidth="1" min="14" max="14"/>
     <col width="8" customWidth="1" min="15" max="15"/>
     <col width="9" customWidth="1" min="16" max="16"/>
-    <col width="8" customWidth="1" min="17" max="17"/>
+    <col width="9" customWidth="1" min="17" max="17"/>
     <col width="62" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
@@ -29735,12 +29735,12 @@
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>Points</t>
+          <t>2026 Proj Pts</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>2025 Exp</t>
+          <t>2025 Pts</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
@@ -29755,7 +29755,7 @@
       </c>
       <c r="Q2" s="2" t="inlineStr">
         <is>
-          <t>Conf</t>
+          <t>Conf Lvl</t>
         </is>
       </c>
       <c r="R2" s="2" t="inlineStr">
@@ -31564,11 +31564,11 @@
     <col width="6" customWidth="1" min="10" max="10"/>
     <col width="7" customWidth="1" min="11" max="11"/>
     <col width="6" customWidth="1" min="12" max="12"/>
-    <col width="9" customWidth="1" min="13" max="13"/>
+    <col width="11" customWidth="1" min="13" max="13"/>
     <col width="10" customWidth="1" min="14" max="14"/>
     <col width="8" customWidth="1" min="15" max="15"/>
     <col width="9" customWidth="1" min="16" max="16"/>
-    <col width="8" customWidth="1" min="17" max="17"/>
+    <col width="9" customWidth="1" min="17" max="17"/>
     <col width="62" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
@@ -31642,12 +31642,12 @@
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>Points</t>
+          <t>2026 Proj Pts</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>2025 Exp</t>
+          <t>2025 Pts</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
@@ -31662,7 +31662,7 @@
       </c>
       <c r="Q2" s="2" t="inlineStr">
         <is>
-          <t>Conf</t>
+          <t>Conf Lvl</t>
         </is>
       </c>
       <c r="R2" s="2" t="inlineStr">
@@ -33607,11 +33607,11 @@
     <col width="6" customWidth="1" min="10" max="10"/>
     <col width="7" customWidth="1" min="11" max="11"/>
     <col width="6" customWidth="1" min="12" max="12"/>
-    <col width="9" customWidth="1" min="13" max="13"/>
+    <col width="11" customWidth="1" min="13" max="13"/>
     <col width="10" customWidth="1" min="14" max="14"/>
     <col width="8" customWidth="1" min="15" max="15"/>
     <col width="9" customWidth="1" min="16" max="16"/>
-    <col width="8" customWidth="1" min="17" max="17"/>
+    <col width="9" customWidth="1" min="17" max="17"/>
     <col width="62" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
@@ -33685,12 +33685,12 @@
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>Points</t>
+          <t>2026 Proj Pts</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>2025 Exp</t>
+          <t>2025 Pts</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
@@ -33705,7 +33705,7 @@
       </c>
       <c r="Q2" s="2" t="inlineStr">
         <is>
-          <t>Conf</t>
+          <t>Conf Lvl</t>
         </is>
       </c>
       <c r="R2" s="2" t="inlineStr">

</xml_diff>